<commit_message>
Update live morning scrape for 05 Oct (3 records)
</commit_message>
<xml_diff>
--- a/EXECUTIVE_TEAM_AUDIT_REPORT_05_Oct_2026.xlsx
+++ b/EXECUTIVE_TEAM_AUDIT_REPORT_05_Oct_2026.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -80,19 +77,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -112,23 +103,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -504,60 +486,78 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Employee Name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Total Scraped Tickets</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Solved / Handled Count</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Solution Rate %</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>GRAND TOTAL (ALL TEAM)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="B4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -583,50 +583,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Task / Issue Type</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Total_Tickets</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Solved_Count</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Solution Rate %</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>% Share of Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>WiFi 6 Upgrade</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>33.3%</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -643,55 +643,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sub Category</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Router Upgrade  Wi-Fi 6</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="6" t="n">
-        <v>2</v>
+      <c r="D2" s="4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -705,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX3"/>
+  <dimension ref="A1:AX4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -739,10 +751,10 @@
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="45" customWidth="1" min="31" max="31"/>
-    <col width="24" customWidth="1" min="32" max="32"/>
+    <col width="25" customWidth="1" min="32" max="32"/>
     <col width="26" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
     <col width="17" customWidth="1" min="36" max="36"/>
     <col width="17" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -751,7 +763,7 @@
     <col width="27" customWidth="1" min="41" max="41"/>
     <col width="12" customWidth="1" min="42" max="42"/>
     <col width="17" customWidth="1" min="43" max="43"/>
-    <col width="34" customWidth="1" min="44" max="44"/>
+    <col width="45" customWidth="1" min="44" max="44"/>
     <col width="34" customWidth="1" min="45" max="45"/>
     <col width="33" customWidth="1" min="46" max="46"/>
     <col width="32" customWidth="1" min="47" max="47"/>
@@ -761,652 +773,880 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Target Employee</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Grid Date</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Grid User Name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Grid Employee Name</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Grid Module</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Grid Operation</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Grid IP Address</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Grid Remark</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Ticket Number</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Account Name</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Case Origin</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Customer Name</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Mobile No</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Sub Sub Category</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Assigned Date</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Estimated closed time based on SLA</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Estimated closed time based on TAT</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>User Id</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Created Date</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Last Modified Date</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Associated Location Status</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Case Reason</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Assign Team</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Assign User</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Customer Address</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Sub Category</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Escalated Layer</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>SLA Left/Total</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>TAT Left/Total</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Last Modified By</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Associated Location Level</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Associated Location Name</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Solution Given</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Employee Remark / Solution Note</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Resolution Time (From Assigned)</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Resolution Time (From Created)</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Resolution Type</t>
         </is>
       </c>
-      <c r="AV1" s="2" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Action / Transfer Remark</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Task / Issue Type</t>
         </is>
       </c>
-      <c r="AX1" s="2" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>Employee Name</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>05 Oct 2026 9:14 AM</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>w7A8I7MXNVw6IhJoudC/TknnOVKMobUO</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 9:55 AM</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>e9R6tm2jVXzJtWahLoJ2dw==</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Case : wifi6  has been updated by Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>wifi6</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>TKT1358080</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Baburaja Maharjan</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>On Hold</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>TKT1356816</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Bishal Regmi</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Baburaja Maharjan</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="n">
-        <v>9841479122</v>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Bishal Regmi</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>9841932852</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>05 Oct 2026 09:14:22 AM</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr"/>
-      <c r="T2" s="3" t="inlineStr"/>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>9841479122</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>04 Oct 2026 02:29:39 PM</t>
-        </is>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>05 Oct 2026 09:14:22 AM</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 09:55:01 AM</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>9841932852</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>03 Oct 2026 04:39:49 PM</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 09:55:01 AM</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="n">
-        <v>27.65564</v>
-      </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>27.75124</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Layer 1-User</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>L1  Support</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr"/>
-      <c r="AE2" s="3" t="inlineStr">
-        <is>
-          <t>27.65564, 85.3402, New Ganesh Temple Naya Basti, M84Q+9V5, Mahalaxmi 44700, Bagmati, Central, Nepal</t>
-        </is>
-      </c>
-      <c r="AF2" s="3" t="inlineStr"/>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>Near Grande Villa,Tokha, Bagmati, Central, Nepal</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>rgmibishal55@gmail.com</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>Router Upgrade  Wi-Fi 6</t>
         </is>
       </c>
-      <c r="AH2" s="3" t="inlineStr"/>
-      <c r="AI2" s="3" t="inlineStr"/>
-      <c r="AJ2" s="3" t="inlineStr"/>
-      <c r="AK2" s="3" t="inlineStr"/>
-      <c r="AL2" s="3" t="inlineStr">
-        <is>
-          <t>Sunita Yonjan</t>
-        </is>
-      </c>
-      <c r="AM2" s="3" t="inlineStr">
-        <is>
-          <t>Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="AN2" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="AO2" s="3" t="inlineStr">
-        <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="AP2" s="3" t="n">
-        <v>85.3402</v>
-      </c>
-      <c r="AQ2" s="3" t="inlineStr"/>
-      <c r="AR2" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="AS2" s="3" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>03:21 hour</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AK2" s="2" t="inlineStr"/>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>Ishlok Shahi</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>L3-1</t>
+        </is>
+      </c>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>85.32164</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr"/>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
         <is>
           <t>0m</t>
         </is>
       </c>
-      <c r="AT2" s="3" t="inlineStr">
-        <is>
-          <t>18h 44m</t>
-        </is>
-      </c>
-      <c r="AU2" s="3" t="inlineStr">
-        <is>
-          <t>Other / In Progress (On Hold)</t>
-        </is>
-      </c>
-      <c r="AV2" s="3" t="inlineStr">
-        <is>
-          <t>Case : wifi6  has been updated by Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="AW2" s="3" t="inlineStr">
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>1d 17h 15m</t>
+        </is>
+      </c>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>Completed (Completed)</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="AW2" s="2" t="inlineStr">
         <is>
           <t>WiFi 6 Upgrade</t>
         </is>
       </c>
-      <c r="AX2" s="3" t="inlineStr">
-        <is>
-          <t>Shashikant Chaudhary</t>
+      <c r="AX2" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 9:14 AM</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>w7A8I7MXNVw6IhJoudC/TknnOVKMobUO</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>wifi6</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>TKT1358080</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Baburaja Maharjan</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>On Hold</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Baburaja Maharjan</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>9841479122</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>General / Other Issues</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 09:14:22 AM</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>9841479122</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>04 Oct 2026 02:29:39 PM</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>05 Oct 2026 09:14:22 AM</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>27.65564</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>General / Other Issues</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>Layer 1-User</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>L1  Support</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>27.65564, 85.3402, New Ganesh Temple Naya Basti, M84Q+9V5, Mahalaxmi 44700, Bagmati, Central, Nepal</t>
+        </is>
+      </c>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Router Upgrade  Wi-Fi 6</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AK3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>Sunita Yonjan</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr">
+        <is>
+          <t>85.3402</t>
+        </is>
+      </c>
+      <c r="AQ3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="AS3" s="2" t="inlineStr">
+        <is>
+          <t>0m</t>
+        </is>
+      </c>
+      <c r="AT3" s="2" t="inlineStr">
+        <is>
+          <t>18h 44m</t>
+        </is>
+      </c>
+      <c r="AU3" s="2" t="inlineStr">
+        <is>
+          <t>Other / In Progress (On Hold)</t>
+        </is>
+      </c>
+      <c r="AV3" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi6  has been updated by Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="AW3" s="2" t="inlineStr">
+        <is>
+          <t>WiFi 6 Upgrade</t>
+        </is>
+      </c>
+      <c r="AX3" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>05 Oct 2026 9:09 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>w7A8I7MXNVw6IhJoudC/TknnOVKMobUO</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Case : Wifi 6   has been updated by Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Wifi 6</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>TKT1357958</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Dinesh Agrawal</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>On Hold</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Dinesh Agrawal</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n">
-        <v>9801172900</v>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>9801172900</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr"/>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>04 Oct 2026 01:33:21 PM</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr"/>
-      <c r="T3" s="3" t="inlineStr"/>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>LTP9705346755</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>04 Oct 2026 01:33:21 PM</t>
         </is>
       </c>
-      <c r="W3" s="3" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>05 Oct 2026 09:09:33 AM</t>
         </is>
       </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr"/>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>Layer 1-User</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
+      <c r="AB4" s="2" t="inlineStr">
         <is>
           <t>Laxman Koirala</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="inlineStr">
+      <c r="AC4" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AD3" s="3" t="inlineStr"/>
-      <c r="AE3" s="3" t="inlineStr">
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr">
         <is>
           <t>Imadol Imadol, Kathmandu, Nepal, Nepal</t>
         </is>
       </c>
-      <c r="AF3" s="3" t="inlineStr">
+      <c r="AF4" s="2" t="inlineStr">
         <is>
           <t>kclalita910@gmail.com</t>
         </is>
       </c>
-      <c r="AG3" s="3" t="inlineStr">
+      <c r="AG4" s="2" t="inlineStr">
         <is>
           <t>Router Upgrade  Wi-Fi 6</t>
         </is>
       </c>
-      <c r="AH3" s="3" t="inlineStr"/>
-      <c r="AI3" s="3" t="inlineStr"/>
-      <c r="AJ3" s="3" t="inlineStr"/>
-      <c r="AK3" s="3" t="inlineStr"/>
-      <c r="AL3" s="3" t="inlineStr">
+      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AK4" s="2" t="inlineStr"/>
+      <c r="AL4" s="2" t="inlineStr">
         <is>
           <t>Sandesh Ghale</t>
         </is>
       </c>
-      <c r="AM3" s="3" t="inlineStr">
+      <c r="AM4" s="2" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="AN3" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO3" s="3" t="inlineStr">
+      <c r="AN4" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO4" s="2" t="inlineStr">
         <is>
           <t>L43-6</t>
         </is>
       </c>
-      <c r="AP3" s="3" t="inlineStr"/>
-      <c r="AQ3" s="3" t="inlineStr"/>
-      <c r="AR3" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="AS3" s="3" t="inlineStr">
+      <c r="AP4" s="2" t="inlineStr"/>
+      <c r="AQ4" s="2" t="inlineStr"/>
+      <c r="AR4" s="2" t="inlineStr">
+        <is>
+          <t>Case : Wifi 6   has been updated by Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="AS4" s="2" t="inlineStr">
         <is>
           <t>19h 36m</t>
         </is>
       </c>
-      <c r="AT3" s="3" t="inlineStr">
+      <c r="AT4" s="2" t="inlineStr">
         <is>
           <t>19h 36m</t>
         </is>
       </c>
-      <c r="AU3" s="3" t="inlineStr">
+      <c r="AU4" s="2" t="inlineStr">
         <is>
           <t>Other / In Progress (On Hold)</t>
         </is>
       </c>
-      <c r="AV3" s="3" t="inlineStr">
+      <c r="AV4" s="2" t="inlineStr">
         <is>
           <t>Case : Wifi 6   has been updated by Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="AW3" s="3" t="inlineStr">
+      <c r="AW4" s="2" t="inlineStr">
         <is>
           <t>WiFi 6 Upgrade</t>
         </is>
       </c>
-      <c r="AX3" s="3" t="inlineStr">
+      <c r="AX4" s="2" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>

</xml_diff>